<commit_message>
Add speaker name label on dialogue bubbles
Name sits on the bubble's top edge at the tail side. Color comes from
the new optional Characters.name_color column (#RRGGBB).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -506,7 +506,6 @@
           <t>t1_intro</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>t1_timeout</t>
@@ -630,7 +629,6 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>노드 0 (도입, 선택지 없음 → 계속)</t>
@@ -668,8 +666,6 @@
           <t>노드 A (조건부 선택지 테스트)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -682,14 +678,11 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>노드 B (탐색·인벤토리 테스트)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -734,14 +727,11 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>노드 D (결말·스탯 테스트)</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -754,7 +744,6 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>시간 초과 노드</t>
@@ -765,7 +754,6 @@
           <t>END:end_t1_timeout</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -788,8 +776,6 @@
           <t>노드 A (에피소드 2)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -802,7 +788,6 @@
           <t>ep_test2</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>시간 초과 노드 (에피소드 2)</t>
@@ -813,7 +798,6 @@
           <t>END:end_t2_timeout</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -897,10 +881,6 @@
           <t>선택지 1 (일반)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>t1_b</t>
@@ -933,8 +913,6 @@
           <t>gray</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>t1_c</t>
@@ -967,8 +945,6 @@
           <t>hide</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>t1_c</t>
@@ -991,8 +967,6 @@
           <t>선택지 4 (대가형)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>체력 -10, 시간 -10</t>
@@ -1025,8 +999,6 @@
           <t>탐색 (spot_b)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>시간 -10</t>
@@ -1059,8 +1031,6 @@
           <t>빈 곳 탐색 (spot_empty)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>시간 -5</t>
@@ -1093,9 +1063,6 @@
           <t>잡동사니 9개 줍기 (인벤토리 초과)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>item:+junk*9</t>
@@ -1123,10 +1090,6 @@
           <t>노드 A로</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>t1_a</t>
@@ -1149,10 +1112,6 @@
           <t>정상 클리어</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>END:end_t1_clear</t>
@@ -1185,8 +1144,6 @@
           <t>gray</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>END:end_t1_good</t>
@@ -1219,7 +1176,6 @@
           <t>hide</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>item:+pill</t>
@@ -1289,8 +1245,6 @@
           <t>사망 테스트</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>체력 -999</t>
@@ -1323,8 +1277,6 @@
           <t>광기 테스트</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>정신력 -999</t>
@@ -1357,8 +1309,6 @@
           <t>시간 초과 테스트</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>시간 -999</t>
@@ -1391,10 +1341,6 @@
           <t>클리어</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>END:end_t2_clear</t>
@@ -1417,8 +1363,6 @@
           <t>시간 초과 테스트</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>시간 -999</t>
@@ -1540,7 +1484,6 @@
           <t>아이템 설명 2</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
         <v>1</v>
       </c>
@@ -1566,7 +1509,6 @@
           <t>아이템 설명 3</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
         <v>1</v>
       </c>
@@ -1744,12 +1686,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.8" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="11.6" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1768,6 +1711,11 @@
           <t>traits</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>name_color</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1785,6 +1733,11 @@
           <t>tester</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>#D81B4A</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1797,7 +1750,6 @@
           <t>주인공 2</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1810,7 +1762,11 @@
           <t>NPC 1</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>#F2C200</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1893,7 +1849,6 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1906,7 +1861,6 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1919,7 +1873,6 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1949,7 +1902,6 @@
           <t>ep_test2</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1962,7 +1914,6 @@
           <t>ep_test2</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1975,7 +1926,6 @@
           <t>ep_test2</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2129,7 +2079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -2142,9 +2092,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -2180,9 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -2225,9 +2171,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -2267,6 +2211,13 @@
       <c r="A21" t="inlineStr">
         <is>
           <t>표에 없는 열(메모 등)을 추가해도 변환 시 무시된다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Characters.name_color: 대화 이름표 색 (#RRGGBB). 비우면 기본색.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dialogue placement: NPCs fill left then right, protagonist is tail-less
- Protagonist lines: no portrait, no name label, bubble without tail
- First NPC to speak takes the left slot, the next one the right slot
- Portraits dim only while the other NPC is speaking
- ep_test2 now opens with an NPC 1 -> NPC 2 exchange to cover the 2-NPC case

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -540,7 +540,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>t2_a</t>
+          <t>t2_npc1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,62 @@
           <t>END:end_t2_timeout</t>
         </is>
       </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>t2_npc1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ep_test2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>char_npc</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>노드 N1 (NPC 1 대사)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>t2_npc2</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>t2_npc2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ep_test2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>char_npc2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>노드 N2 (NPC 2 대사)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>t2_a</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1686,7 +1742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.8" customWidth="1" min="1" max="1"/>
@@ -1765,6 +1821,24 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>#F2C200</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>char_npc2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NPC 2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>#4FC3F7</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2166,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -2128,7 +2201,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -2171,7 +2243,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Converter: abilities, dice choices, item dice bonuses
- Optional Abilities sheet; Characters.abilities base values
- Choices.type normal/item/dice with check, dc, mod, fail_effects, fail_next
- Items.dice_bonus; condition abil:x>=n and effect abil:x+n
- Dummy dice test node t1_e in ep_test1

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -14,8 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loot" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Characters" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endings" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abilities" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -569,13 +570,215 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="90" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>문법 요약 (이 시트는 변환 시 무시됨: 이름이 _로 시작)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>[조건] &amp; = AND, | = OR, ! = NOT, 괄호 () 사용 가능. 우선순위: ! &gt; &amp; &gt; |</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>has:knife  /  has:bandage&gt;=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>flag:door_open (에피소드 플래그)  /  wflag:ep1_clear (월드 플래그)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>stat:sanity&gt;=30   (비교: &gt; &gt;= &lt; &lt;= ==, 스탯: hp sanity time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>trait:medic (현재 주인공 능력)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>[효과] ; 로 구분</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>item:+bandage  /  item:-bandage  /  item:+bandage*2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>stat:hp-10  /  stat:hp+10  /  stat:hp=50</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>setflag:x  /  clearflag:x  /  setwflag:x</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>loot:spot_id (Loot 시트 확률 굴림, chance는 0~100 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>goto:node_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>[진행] 선택지 없는 노드는 next_node로 진행. END:&lt;ending_id&gt; 는 엔딩.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>show_mode: hide(조건 미충족 시 숨김) / gray(회색, 기본값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>cost 는 표시용. 실제 차감은 effects 에 적는다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>아이템 사용 시 소모도 use_effects 에 명시 (예: item:-bandage;stat:hp+20).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Traits / world_flags_set 은 쉼표(,)로 여러 개.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>표에 없는 열(메모 등)을 추가해도 변환 시 무시된다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Characters.name_color: 대화 이름표 색 (#RRGGBB). 비우면 기본색.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>[주사위 판정] d20 + 보정치 &gt;= dc 이면 성공. 성공 확률 = (21 - (dc - 보정치)) / 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>보정치 = 능력치(Characters.abilities + abil: 효과로 성장) + 소지 아이템 dice_bonus + 선택지 mod</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Choices.type: normal(기본) / item(condition 에 has: 필요, 가지고 있으면 반드시 성공) / dice</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>dice 선택지: check(능력치) dc(목표값) mod(상황 보정), 성공 → effects·next_node, 실패 → fail_effects·fail_next</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Abilities 시트: ability_id, name.  Characters.abilities: 'stat_a=3, stat_b=1'</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Items.dice_bonus: 'stat_a+2' 또는 'all+1' (소지 중이면 적용, 개수와 무관하게 1번)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>조건 abil:stat_a&gt;=3 / 효과 abil:stat_a+1 (육성)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -825,7 +1028,6 @@
           <t>t2_npc2</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -853,7 +1055,74 @@
           <t>t2_a</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ep_test1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>노드 E (주사위 판정 테스트)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>t1_dice_ok</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ep_test1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>판정 성공 노드</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>t1_dice_fail</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ep_test1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>판정 실패 노드</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -866,7 +1135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.4" customWidth="1" min="1" max="1"/>
@@ -877,6 +1146,12 @@
     <col width="24.4" customWidth="1" min="6" max="6"/>
     <col width="38.8" customWidth="1" min="7" max="7"/>
     <col width="27.6" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -920,6 +1195,36 @@
           <t>next_node</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>dc</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>mod</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>fail_effects</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>fail_next</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -974,6 +1279,11 @@
           <t>t1_c</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1006,6 +1316,11 @@
           <t>t1_c</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1432,6 +1747,222 @@
       <c r="H18" t="inlineStr">
         <is>
           <t>t2_a</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>c_d8</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>t1_d</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>판정 테스트로</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>c_e1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>판정 A (능력치 A, 목표 12)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>setflag:dice_ok</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>t1_dice_ok</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>dice</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>stat_a</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>12</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>stat:hp-5</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>t1_dice_fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>c_e2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>판정 B (능력치 B, 목표 10, 상황 보정 -5)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>t1_dice_ok</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>dice</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>stat_b</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>10</v>
+      </c>
+      <c r="L21" t="n">
+        <v>-5</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>t1_dice_fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>c_e3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>능력치 A 성장 (+1)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>abil:stat_a+1</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>c_e4</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>능력치 조건 (abil:stat_a&gt;=4)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>abil:stat_a&gt;=4</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>c_e5</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>t1_e</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>노드 D로</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>t1_d</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.2" customWidth="1" min="1" max="1"/>
@@ -1455,6 +1986,7 @@
     <col width="19.6" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="16.4" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1488,6 +2020,11 @@
           <t>stack_max</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>dice_bonus</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1542,6 +2079,11 @@
       </c>
       <c r="F3" t="n">
         <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>stat_a+1</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1742,13 +2284,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.8" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="11.6" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1772,6 +2315,11 @@
           <t>name_color</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>abilities</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1794,6 +2342,11 @@
           <t>#D81B4A</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>stat_a=3, stat_b=0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1806,6 +2359,11 @@
           <t>주인공 2</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>stat_a=1, stat_b=2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1835,7 +2393,6 @@
           <t>NPC 2</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>#4FC3F7</t>
@@ -2012,133 +2569,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="19.6" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>ability_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>note</t>
+          <t>name</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>inventory_slots</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>인벤토리 칸 수</t>
+          <t>stat_a</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>능력치 A</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hp_start</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>100</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>에피소드 시작 체력</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>hp_max</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>100</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>체력 최대치</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>sanity_start</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>100</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>에피소드 시작 정신력</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>sanity_max</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>100</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>정신력 최대치</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>time_start</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>120</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>에피소드 시작 시간</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>time_max</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>120</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>시간 최대치</t>
+          <t>stat_b</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>능력치 B</t>
         </is>
       </c>
     </row>
@@ -2153,142 +2623,133 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="19.6" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>문법 요약 (이 시트는 변환 시 무시됨: 이름이 _로 시작)</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>inventory_slots</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>인벤토리 칸 수</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>[조건] &amp; = AND, | = OR, ! = NOT, 괄호 () 사용 가능. 우선순위: ! &gt; &amp; &gt; |</t>
+          <t>hp_start</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>에피소드 시작 체력</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>has:knife  /  has:bandage&gt;=2</t>
+          <t>hp_max</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>체력 최대치</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>flag:door_open (에피소드 플래그)  /  wflag:ep1_clear (월드 플래그)</t>
+          <t>sanity_start</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>에피소드 시작 정신력</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>stat:sanity&gt;=30   (비교: &gt; &gt;= &lt; &lt;= ==, 스탯: hp sanity time)</t>
+          <t>sanity_max</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>정신력 최대치</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>trait:medic (현재 주인공 능력)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>[효과] ; 로 구분</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>item:+bandage  /  item:-bandage  /  item:+bandage*2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>stat:hp-10  /  stat:hp+10  /  stat:hp=50</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>setflag:x  /  clearflag:x  /  setwflag:x</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>loot:spot_id (Loot 시트 확률 굴림, chance는 0~100 %)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>goto:node_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>[진행] 선택지 없는 노드는 next_node로 진행. END:&lt;ending_id&gt; 는 엔딩.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>show_mode: hide(조건 미충족 시 숨김) / gray(회색, 기본값)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>cost 는 표시용. 실제 차감은 effects 에 적는다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>아이템 사용 시 소모도 use_effects 에 명시 (예: item:-bandage;stat:hp+20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Traits / world_flags_set 은 쉼표(,)로 여러 개.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>표에 없는 열(메모 등)을 추가해도 변환 시 무시된다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Characters.name_color: 대화 이름표 색 (#RRGGBB). 비우면 기본색.</t>
+          <t>time_start</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>120</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>에피소드 시작 시간</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>time_max</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>120</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>시간 최대치</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Converter: combat sheets (PlayerParts, Enemies, EnemyParts, EnemyAttacks)
Attack patterns normal/quick/combo/feint are exported as strike lists
({telegraph, target}). Combat tuning lives in Config combat_* keys.
Dummy enemy enemy_test with one attack of each pattern.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -16,7 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endings" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abilities" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerParts" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyParts" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -576,7 +580,625 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>part_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>vital</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>머리</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>몸통</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>50</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>left_arm</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>왼팔</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>right_arm</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>오른팔</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>left_leg</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>왼다리</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>right_leg</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>오른다리</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>enemy_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>적 A (테스트)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>enemy_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>part_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>hit_chance</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>vital</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>머리</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>몸통</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E3" t="n">
+        <v>90</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>left_arm</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>왼팔</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>70</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>right_arm</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>오른팔</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>70</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>attack_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>enemy_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>part</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>targets</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>windup</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>atk_normal</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>일반 공격 (테스트)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>right_arm</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>atk_quick</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>속공 (테스트)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>left_arm</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>quick</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>left_arm</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>atk_combo</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>연속 공격 (테스트)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>right_arm</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>head, right_leg</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>atk_feint</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>기만 공격 (테스트)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>feint</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>torso&gt;head</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H5" t="n">
+        <v>12</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -715,9 +1337,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -764,6 +1384,51 @@
       <c r="A30" t="inlineStr">
         <is>
           <t>조건 abil:stat_a&gt;=3 / 효과 abil:stat_a+1 (육성)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>[전투] PlayerParts: 플레이어 부위 (key = 회피 키 W/A/S/D, vital=Y 면 파괴 시 사망)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Enemies / EnemyParts(적별 부위, hit_chance %) / EnemyAttacks(적 공격)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>EnemyAttacks.pattern: normal / quick / combo(targets 'head, torso' 순서대로) / feint(targets '전조&gt;실제')</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>EnemyAttacks.part: 이 공격을 쓰는 적 부위. 그 부위가 파괴되면 이 공격은 못 씀</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>windup: 전조 시간(초). 이 시간이 끝나는 순간이 회피 타이밍. weight: 공격 선택 가중치</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Config combat_*: 회피 판정 시간, 플레이어 피해, 방어 배율, 도주 확률, 기만 전환 시점</t>
         </is>
       </c>
     </row>
@@ -1067,14 +1732,11 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>노드 E (주사위 판정 테스트)</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1087,7 +1749,6 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>판정 성공 노드</t>
@@ -1098,7 +1759,6 @@
           <t>t1_e</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1111,7 +1771,6 @@
           <t>ep_test1</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>판정 실패 노드</t>
@@ -1122,7 +1781,6 @@
           <t>t1_e</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1766,10 +2424,6 @@
           <t>판정 테스트로</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>t1_e</t>
@@ -1792,9 +2446,6 @@
           <t>판정 A (능력치 A, 목표 12)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>setflag:dice_ok</t>
@@ -1845,10 +2496,6 @@
           <t>판정 B (능력치 B, 목표 10, 상황 보정 -5)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>t1_dice_ok</t>
@@ -1892,9 +2539,6 @@
           <t>능력치 A 성장 (+1)</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>abil:stat_a+1</t>
@@ -1932,8 +2576,6 @@
           <t>gray</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>t1_e</t>
@@ -1956,10 +2598,6 @@
           <t>노드 D로</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>t1_d</t>
@@ -2623,7 +3261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2753,6 +3391,96 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>combat_perfect_window</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>완벽 회피 허용 오차 (초, ±)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>combat_normal_window</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>일반 회피 허용 오차 (초, ±)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>combat_player_damage</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>플레이어 공격 피해</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>combat_defend_mult</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>방어 시 받는 피해 배율</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>combat_flee_chance</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>50</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>도주 성공 확률 (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>combat_feint_switch</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>기만 공격 전조가 바뀌는 시점 (전조 시간 비율)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Converter: text maps (tools/maps/*.txt) and FieldObjects sheet
Maps use # wall, . floor, P start and single-letter markers that refer
to FieldObjects rows (enemy with patrol, investigate with optional loot).
Field tuning in Config field_* keys. Dummy map test_field.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -20,7 +20,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyParts" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldObjects" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -686,7 +687,6 @@
       <c r="D4" t="n">
         <v>25</v>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -707,7 +707,6 @@
       <c r="D5" t="n">
         <v>25</v>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -728,7 +727,6 @@
       <c r="D6" t="n">
         <v>25</v>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -749,7 +747,6 @@
       <c r="D7" t="n">
         <v>25</v>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -925,7 +922,6 @@
       <c r="E4" t="n">
         <v>70</v>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -949,7 +945,6 @@
       <c r="E5" t="n">
         <v>70</v>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1198,7 +1193,259 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>object_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>map_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>marker</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ref</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>patrol</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>fo_enemy1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>적 A (테스트)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>right 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>fo_enemy2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>enemy_test</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>적 A (테스트)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>down 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fo_look1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>investigate</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>spot_b</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>조사 지점 1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>조사 텍스트 1 (테스트)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>fo_look2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>investigate</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>조사 지점 2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>조사 텍스트 2 (테스트, 아이템 없음)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>fo_look3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>investigate</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>spot_empty</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>조사 지점 3</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>조사 텍스트 3 (테스트, 빈 탐색)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1337,7 +1584,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -1387,9 +1633,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -1429,6 +1673,30 @@
       <c r="A37" t="inlineStr">
         <is>
           <t>Config combat_*: 회피 판정 시간, 플레이어 피해, 방어 배율, 도주 확률, 기만 전환 시점</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>[탐험] 맵 모양: tools/maps/&lt;map_id&gt;.txt  (# 벽, . 바닥, P 시작 위치, 그 밖의 글자 = FieldObjects 의 marker)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>FieldObjects: type enemy(ref=enemy_id, patrol='right 4' 처럼 방향+칸수 왕복) / investigate(text 표시, ref=Loot spot_id 면 아이템 굴림)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Config field_*: 칸 크기, 이동·순찰·추격 속도, 시야, 추격 포기 거리, 도주 후 유예 시간</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3481,6 +3749,111 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>field_tile</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>48</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>탐험 맵 한 칸 크기 (픽셀)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>field_player_speed</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>플레이어 이동 속도 (칸/초)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>field_enemy_speed</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>적 순찰 속도 (칸/초)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>field_enemy_chase_speed</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>적 추격 속도 (칸/초)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>field_enemy_sight</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>적 시야 (칸). 벽 너머는 못 봄</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>field_enemy_lose_sight</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>이 거리 넘게 멀어지면 추격 포기 (칸)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>field_flee_grace</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>도주 후 적이 다시 덤비지 않는 시간 (초)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Converter: field dialogue nodes (empty episode_id, EXIT) and npc objects
- Nodes without episode_id are field dialogue; EXIT ends the dialogue
- FieldObjects type=npc refers to a field dialogue start node
- Config accepts string values; protagonist_id names the field protagonist
- Dummy NPC 1 (normal/item/dice choices) and NPC 2 (flag-gated line)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -1193,7 +1193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1279,7 +1279,6 @@
           <t>적 A (테스트)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>right 5</t>
@@ -1317,7 +1316,6 @@
           <t>적 A (테스트)</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>down 3</t>
@@ -1360,7 +1358,6 @@
           <t>조사 텍스트 1 (테스트)</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1383,7 +1380,6 @@
           <t>investigate</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>조사 지점 2</t>
@@ -1394,7 +1390,6 @@
           <t>조사 텍스트 2 (테스트, 아이템 없음)</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1432,7 +1427,74 @@
           <t>조사 텍스트 3 (테스트, 빈 탐색)</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fo_npc1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>npc</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>fd_npc1_a</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NPC 1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fo_npc2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>npc</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>fd_npc2_a</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>NPC 2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1445,7 +1507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1633,7 +1695,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -1676,9 +1737,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
@@ -1697,6 +1756,30 @@
       <c r="A41" t="inlineStr">
         <is>
           <t>Config field_*: 칸 크기, 이동·순찰·추격 속도, 시야, 추격 포기 거리, 도주 후 유예 시간</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>[필드 대화] Nodes 에서 episode_id 를 비운 노드 = 필드 대화. 대화를 끝낼 때 next_node(또는 fail_next)에 EXIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>FieldObjects type=npc, ref=필드 대화 시작 노드. 말을 걸 때마다 시작 노드부터 (조건·플래그로 내용 분기)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Config protagonist_id: 탐험 중 주인공 (능력치·능력·주사위 보정)</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2050,6 +2133,118 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>fd_npc1_a</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>char_npc</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>필드 대화 노드 1 (NPC 1)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>fd_npc1_b</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>char_t1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>필드 대화 노드 2 (주인공)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>fd_npc1_fail</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>char_npc</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>필드 대화 노드 3 (판정 실패)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>fd_npc2_a</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>char_npc2</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>필드 대화 노드 4 (NPC 2)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>fd_npc2_b</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>char_npc2</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>필드 대화 노드 5 (flag:showed_knife 일 때만)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2061,7 +2256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.4" customWidth="1" min="1" max="1"/>
@@ -2869,6 +3064,209 @@
       <c r="H24" t="inlineStr">
         <is>
           <t>t1_d</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>fdc1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>fd_npc1_a</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>대화 선택지 1 (일반)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>fd_npc1_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>fdc2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>fd_npc1_a</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>칼 보여주기</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>has:knife</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>setflag:showed_knife</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>fd_npc1_b</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>fdc3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>fd_npc1_a</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>설득 (능력치 A, 목표 12)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>item:+bandage</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>fd_npc1_b</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>dice</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>stat_a</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>12</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>fd_npc1_fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>fdc4</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>fd_npc1_a</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>대화 끝내기</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>fdc5</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>fd_npc2_a</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>칼 이야기 (flag:showed_knife)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>flag:showed_knife</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>hide</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>fd_npc2_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>fdc6</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>fd_npc2_a</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>대화 끝내기</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>EXIT</t>
         </is>
       </c>
     </row>
@@ -3529,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3854,6 +4252,23 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>protagonist_id</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>char_t1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>주인공 char_id (탐험·필드 대화의 능력치·능력·대화 배치)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Converter: survival params, camp actions, basecamp map, map exits
- Survival sheet (start, max, decay per hour, warn) and surv: grammar
- CampActions sheet (minutes, condition, effects, kind=save)
- FieldObjects camp/exit; Config start_map, basecamp_map, time_scale, start_hour
- Dummy basecamp map linked to test_field, food/water items and supply spot

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -21,7 +21,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyParts" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldObjects" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survival" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampActions" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1193,7 +1195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1459,8 +1461,6 @@
           <t>NPC 1</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1493,8 +1493,142 @@
           <t>NPC 2</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>fo_camp</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>basecamp</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>camp</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>베이스캠프 거점</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>fo_to_field</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>basecamp</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>탐험 지역으로</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>fo_to_camp</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>basecamp</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>베이스캠프로</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>fo_supply</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>test_field</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>investigate</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>spot_supply</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>보급 상자</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>조사 텍스트 4 (테스트, 음식·물)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1507,7 +1641,375 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>param_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>decay_per_hour</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>hunger</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>포만감</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>80</v>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>thirst</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>수분</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>80</v>
+      </c>
+      <c r="D3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sleep</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>수면</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>90</v>
+      </c>
+      <c r="D4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>hygiene</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>위생</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>90</v>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>mental</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>멘탈</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>action_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>minutes</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>effects</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>camp_eat</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>식사 (통조림 1개)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>has:food</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>item:-food;surv:hunger+50</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>camp_drink</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>물 마시기 (물 1병)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>has:water</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>item:-water;surv:thirst+60</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>camp_sleep4</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>수면 (4시간)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>240</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>surv:sleep+40</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>camp_sleep8</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>수면 (8시간)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>480</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>surv:sleep+80;surv:mental+10</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>camp_wash</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>씻기</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>surv:hygiene+60</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>camp_save</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>저장</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>save</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1737,7 +2239,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
@@ -1759,9 +2260,7 @@
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-    </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
@@ -1780,6 +2279,44 @@
       <c r="A45" t="inlineStr">
         <is>
           <t>Config protagonist_id: 탐험 중 주인공 (능력치·능력·주사위 보정)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>[생존] Survival: 파라미터 (100 = 좋음, 0 = 최악). decay_per_hour = 게임 1시간마다 줄어드는 양, warn = 경고 표시 기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>조건 surv:hunger&lt;30 / 효과 surv:hunger+40</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>[베이스캠프] CampActions: 베이스캠프 거점(FieldObjects type=camp)에서 고르는 행동. minutes = 걸리는 시간, kind=save 는 저장</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>FieldObjects type=exit: ref = 이동할 맵 이름. 도착하면 그 맵의 P 위치</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Config start_map / basecamp_map / time_scale(실제 1초 = 게임 몇 분) / start_hour</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2676,6 @@
           <t>fd_npc1_a</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>char_npc</t>
@@ -2150,8 +2686,6 @@
           <t>필드 대화 노드 1 (NPC 1)</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2159,7 +2693,6 @@
           <t>fd_npc1_b</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>char_t1</t>
@@ -2175,7 +2708,6 @@
           <t>EXIT</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2183,7 +2715,6 @@
           <t>fd_npc1_fail</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>char_npc</t>
@@ -2199,7 +2730,6 @@
           <t>EXIT</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2207,7 +2737,6 @@
           <t>fd_npc2_a</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>char_npc2</t>
@@ -2218,8 +2747,6 @@
           <t>필드 대화 노드 4 (NPC 2)</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2227,7 +2754,6 @@
           <t>fd_npc2_b</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>char_npc2</t>
@@ -2243,7 +2769,6 @@
           <t>EXIT</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3083,10 +3608,6 @@
           <t>대화 선택지 1 (일반)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>fd_npc1_b</t>
@@ -3119,7 +3640,6 @@
           <t>gray</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>setflag:showed_knife</t>
@@ -3152,9 +3672,6 @@
           <t>설득 (능력치 A, 목표 12)</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>item:+bandage</t>
@@ -3200,10 +3717,6 @@
           <t>대화 끝내기</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>EXIT</t>
@@ -3236,8 +3749,6 @@
           <t>hide</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>fd_npc2_b</t>
@@ -3260,10 +3771,6 @@
           <t>대화 끝내기</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>EXIT</t>
@@ -3281,7 +3788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.2" customWidth="1" min="1" max="1"/>
@@ -3445,6 +3952,66 @@
         <v>3</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>통조림(테스트)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>아이템 설명 5</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>item:-food;surv:hunger+40</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>물(테스트)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>drink</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>아이템 설명 6</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>item:-water;surv:thirst+50</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3456,7 +4023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.2" customWidth="1" min="1" max="1"/>
@@ -3575,6 +4142,58 @@
       </c>
       <c r="F4" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>l4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>spot_supply</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>l5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>spot_supply</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3927,7 +4546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4269,6 +4888,70 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>start_map</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>basecamp</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>새 회차를 시작하는 맵</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>basecamp_map</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>basecamp</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>베이스캠프 맵 (저장 가능한 유일한 곳)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>time_scale</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>탐험 중 실제 1초에 흐르는 게임 시간 (분)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>start_hour</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>새 회차 시작 시각 (시)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Survival and basecamp in the field; run-based title
- Field: real-time clock and survival HUD, inventory (I/Tab) with item
  use, investigate via StoryRunner (discard prompt when full, time cost)
- Basecamp map with camp menu (eat, drink, sleep, wash, save) and exits
  between maps; maps rebuild in place from run state
- Death ends the run (save deleted); new run restarts at basecamp
- Title: new run / continue (last basecamp save) / prototype tests
- basecamp_smoke covers camp actions, save, travel, time, eating, continue

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -1515,14 +1515,11 @@
           <t>camp</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>베이스캠프 거점</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1555,8 +1552,6 @@
           <t>탐험 지역으로</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1589,8 +1584,6 @@
           <t>베이스캠프로</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1628,7 +1621,6 @@
           <t>조사 텍스트 4 (테스트, 음식·물)</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1882,7 +1874,6 @@
           <t>item:-food;surv:hunger+50</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1908,7 +1899,6 @@
           <t>item:-water;surv:thirst+60</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1918,19 +1908,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>수면 (4시간)</t>
+          <t>짧게 자기</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>240</v>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>surv:sleep+40</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1940,19 +1928,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>수면 (8시간)</t>
+          <t>푹 자기</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>480</v>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>surv:sleep+80;surv:mental+10</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1968,13 +1954,11 @@
       <c r="C6" t="n">
         <v>30</v>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>surv:hygiene+60</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1990,8 +1974,6 @@
       <c r="C7" t="n">
         <v>0</v>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>save</t>
@@ -2260,7 +2242,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
@@ -2282,9 +2263,7 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-    </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Data: cat NPC save, hourly sleep that saves, object conditions
- Effect 'save' saves the run (basecamp only, checked at runtime)
- CampActions kind=sleep (1-hour units, effects per hour); the separate
  save action and fixed 4h/8h sleeps are replaced by one hourly sleep
- FieldObjects.condition: object appears only when true (cat presence)
- Dummy cat NPC at basecamp with a 'pet (save)' choice

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -1195,7 +1195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1206,6 +1206,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1249,6 +1250,11 @@
           <t>patrol</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1619,6 +1625,45 @@
       <c r="G12" t="inlineStr">
         <is>
           <t>조사 텍스트 4 (테스트, 음식·물)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>fo_cat</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>basecamp</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>npc</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>fd_cat_a</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>고양이</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>!wflag:cat_away</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1903,80 +1948,46 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>camp_sleep4</t>
+          <t>camp_wash</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>짧게 자기</t>
+          <t>씻기</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>240</v>
+        <v>30</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>surv:sleep+40</t>
+          <t>surv:hygiene+60</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>camp_sleep8</t>
+          <t>camp_sleep</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>푹 자기</t>
+          <t>잠자기</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>480</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>surv:sleep+80;surv:mental+10</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>camp_wash</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>씻기</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>surv:hygiene+60</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>camp_save</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>저장</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>save</t>
+          <t>surv:sleep+10</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>sleep</t>
         </is>
       </c>
     </row>
@@ -1991,7 +2002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A51"/>
+  <dimension ref="A1:A56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -2263,7 +2274,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
@@ -2296,6 +2306,37 @@
       <c r="A51" t="inlineStr">
         <is>
           <t>Config start_map / basecamp_map / time_scale(실제 1초 = 게임 몇 분) / start_hour</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>[저장] 베이스캠프에서만. 고양이(FieldObjects condition 이 참일 때만 나타남)에게 효과 save 로 저장하거나, 잠자기(CampActions kind=sleep)로 자고 나면 저장</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>효과 save: 회차 저장 (베이스캠프 밖에서는 '여기서는 저장할 수 없다')</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CampActions kind=sleep: minutes=60, effects 는 1시간마다 적용, 1~sleep_max_hours 시간 중 골라 잔다</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>FieldObjects.condition: 맵에 들어올 때 참이어야 물체가 나타남 (비우면 항상)</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2749,6 +2790,26 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>fd_cat_a</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>char_cat</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>고양이 노드 (테스트, 사람 말을 하지 않는다)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2760,7 +2821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.4" customWidth="1" min="1" max="1"/>
@@ -3751,6 +3812,62 @@
         </is>
       </c>
       <c r="H30" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fdc_cat1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>fd_cat_a</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>쓰다듬는다 (저장)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>save</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>fdc_cat2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>fd_cat_a</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>그냥 둔다</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
         <is>
           <t>EXIT</t>
         </is>
@@ -4186,7 +4303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.8" customWidth="1" min="1" max="1"/>
@@ -4300,6 +4417,25 @@
           <t>#4FC3F7</t>
         </is>
       </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>char_cat</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>고양이</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>#E8B04A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4525,7 +4661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4931,6 +5067,21 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>sleep_max_hours</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>12</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>한 번에 잘 수 있는 최대 시간</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
NPC daily routines (FieldObjects.schedule); sleep saves even with the cat
- schedule column: time ranges like '06:00-12:00, 20:00-23:00' (past
  midnight allowed); NPCs appear/disappear live as the clock moves
- Dummy cat routine 06:00-12:00, 20:00-23:00 replaces the flag condition
- Sleep always saves (confirmed); camp menu shows '잠자기 (1시간 단위)'
- Tests: schedule ranges, cat leaving at 16h and returning at 20h

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -1195,7 +1195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1207,6 +1207,7 @@
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1255,6 +1256,11 @@
           <t>condition</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1659,11 +1665,9 @@
           <t>고양이</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>!wflag:cat_away</t>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>06:00-12:00, 20:00-23:00</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1983,6 @@
       <c r="C5" t="n">
         <v>60</v>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>surv:sleep+10</t>
@@ -2002,7 +2005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A56"/>
+  <dimension ref="A1:A57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -2309,9 +2312,6 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-    </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
@@ -2337,6 +2337,13 @@
       <c r="A56" t="inlineStr">
         <is>
           <t>FieldObjects.condition: 맵에 들어올 때 참이어야 물체가 나타남 (비우면 항상)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>FieldObjects.schedule (npc): 하루 중 있는 시간대 '06:00-12:00, 20:00-23:00'. 자정 넘김 '22:00-02:00' 가능. 시간이 흐르면 나타나고 사라짐</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2803,6 @@
           <t>fd_cat_a</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>char_cat</t>
@@ -2807,8 +2813,6 @@
           <t>고양이 노드 (테스트, 사람 말을 하지 않는다)</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3833,9 +3837,6 @@
           <t>쓰다듬는다 (저장)</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>save</t>
@@ -3863,10 +3864,6 @@
           <t>그냥 둔다</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>EXIT</t>
@@ -4429,13 +4426,11 @@
           <t>고양이</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>#E8B04A</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sleep picker: adjust hours with left/right arrows
◀ N시간 ▶ stepper (arrows, A/D, pad left/right, hold to repeat) with
wake-time preview; E/Space/Enter sleeps, Esc cancels. Starts at Config
sleep_default_hours (8), clamped to 1..sleep_max_hours.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -4656,7 +4656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5077,6 +5077,21 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>sleep_default_hours</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>잠자기를 고를 때 처음 표시되는 시간</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Washing at the basecamp needs and uses 1 water
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -1957,15 +1957,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>씻기</t>
+          <t>씻기 (물 1병)</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>30</v>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>has:water</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>surv:hygiene+60</t>
+          <t>item:-water;surv:hygiene+60</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Data: Revivals sheet, run start marker S, start_map = test_field
- Revivals rows (condition, effects, text) decide revival on death
- Map letter S marks where a new run wakes up; P stays the arrival point
- Dummy: revive charm item (spot_charm) and a cat choice granting
  hana_protect

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -23,7 +23,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldObjects" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survival" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampActions" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revivals" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1394,6 +1395,11 @@
           <t>investigate</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>spot_charm</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>조사 지점 2</t>
@@ -1401,7 +1407,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>조사 텍스트 2 (테스트, 아이템 없음)</t>
+          <t>조사 텍스트 2 (테스트, 부활 아이템)</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2016,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A57"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>revive_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>effects</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>rv_charm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>부활 부적</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>has:charm</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>item:-charm</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>부활 텍스트 1 (테스트, 아이템으로 부활)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>rv_hana</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>초월체의 보호</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>flag:hana_protect</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>clearflag:hana_protect</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>부활 텍스트 2 (테스트, 초월체가 부활시킴)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -2349,6 +2457,30 @@
       <c r="A57" t="inlineStr">
         <is>
           <t>FieldObjects.schedule (npc): 하루 중 있는 시간대 '06:00-12:00, 20:00-23:00'. 자정 넘김 '22:00-02:00' 가능. 시간이 흐르면 나타나고 사라짐</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>[부활] Revivals: 사망 순간 위에서부터 condition 이 참인 첫 행으로 부활. effects 적용(예: 아이템 소모), text 표시</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → 소지품·시간·생존·부상·플래그 모두 유지한 채 베이스캠프(P)에서 깨어남. 맞는 행이 없으면 게임 처음부터</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>맵 글자 S: 새 회차 시작 위치 (Config start_map 의 맵). 없으면 P</t>
         </is>
       </c>
     </row>
@@ -2830,7 +2962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.4" customWidth="1" min="1" max="1"/>
@@ -3875,6 +4007,44 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>fdc_cat3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>fd_cat_a</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>(테스트) 부활 보호 받기</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>!flag:hana_protect</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>hide</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>setflag:hana_protect</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3886,7 +4056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.2" customWidth="1" min="1" max="1"/>
@@ -4110,6 +4280,32 @@
         <v>5</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>charm</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>부활 부적(테스트)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>아이템 설명 7</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4121,7 +4317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.2" customWidth="1" min="1" max="1"/>
@@ -4292,6 +4488,32 @@
       </c>
       <c r="F6" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>l6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>spot_charm</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>charm</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5011,12 +5233,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>basecamp</t>
+          <t>test_field</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>새 회차를 시작하는 맵</t>
+          <t>새 회차(첫 시작·부활 없는 사망 후)를 시작하는 맵. 그 맵의 S 위치에서 깨어남</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multiple save slots (5), chosen on every save
- SaveManager: run_<n>.json slots with meta (day, time, run, saved at),
  latest_slot(), migration of the old run.json to slot 1
- ui/save_slot_picker: save mode (overwrite needs a second press, 'don't
  save' option) and load mode; keyboard ↑↓ Enter Esc
- Sleeping and the cat's save effect open the picker; the title's
  Continue opens it in load mode
- Config save_slots = 5

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2118,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:A62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -2460,9 +2460,7 @@
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr"/>
-    </row>
+    <row r="58"/>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
@@ -2481,6 +2479,13 @@
       <c r="A61" t="inlineStr">
         <is>
           <t>맵 글자 S: 새 회차 시작 위치 (Config start_map 의 맵). 없으면 P</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Config save_slots: 저장 슬롯 수. 잠에서 깨거나 효과 save(고양이)로 저장할 때 슬롯을 고름</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4038,6 @@
           <t>hide</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>setflag:hana_protect</t>
@@ -4301,7 +4305,6 @@
           <t>아이템 설명 7</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>1</v>
       </c>
@@ -4883,7 +4886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5319,6 +5322,21 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>save_slots</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>저장 슬롯 수 (저장·이어하기 때 고른다)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Dialogue files: tools/dialogues/*.json as the source for dialogue
The converter merges dialogue files (one per conversation, with node
positions for the editor) after the Excel Nodes/Choices rows and
validates them together; errors point at the file. Field dialogues
(NPC 1, NPC 2, cat) moved out of Excel; converted data is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2460,7 +2460,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
@@ -2500,7 +2499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2839,123 +2838,6 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>fd_npc1_a</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>char_npc</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>필드 대화 노드 1 (NPC 1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>fd_npc1_b</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>char_t1</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>필드 대화 노드 2 (주인공)</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>EXIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>fd_npc1_fail</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>char_npc</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>필드 대화 노드 3 (판정 실패)</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>EXIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>fd_npc2_a</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>char_npc2</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>필드 대화 노드 4 (NPC 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>fd_npc2_b</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>char_npc2</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>필드 대화 노드 5 (flag:showed_knife 일 때만)</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>EXIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>fd_cat_a</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>char_cat</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>고양이 노드 (테스트, 사람 말을 하지 않는다)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2967,7 +2849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.4" customWidth="1" min="1" max="1"/>
@@ -3775,277 +3657,6 @@
       <c r="H24" t="inlineStr">
         <is>
           <t>t1_d</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>fdc1</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>fd_npc1_a</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>대화 선택지 1 (일반)</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>fd_npc1_b</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>fdc2</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>fd_npc1_a</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>칼 보여주기</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>has:knife</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>gray</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>setflag:showed_knife</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>fd_npc1_b</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>item</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>fdc3</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>fd_npc1_a</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>설득 (능력치 A, 목표 12)</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>item:+bandage</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>fd_npc1_b</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>dice</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>stat_a</t>
-        </is>
-      </c>
-      <c r="K27" t="n">
-        <v>12</v>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>fd_npc1_fail</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>fdc4</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>fd_npc1_a</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>대화 끝내기</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>EXIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>fdc5</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>fd_npc2_a</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>칼 이야기 (flag:showed_knife)</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>flag:showed_knife</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>hide</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>fd_npc2_b</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>fdc6</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>fd_npc2_a</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>대화 끝내기</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>EXIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>fdc_cat1</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>fd_cat_a</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>쓰다듬는다 (저장)</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>save</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>EXIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>fdc_cat2</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>fd_cat_a</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>그냥 둔다</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>EXIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>fdc_cat3</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>fd_cat_a</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>(테스트) 부활 보호 받기</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>!flag:hana_protect</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>hide</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>setflag:hana_protect</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>EXIT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Map files: tools/maps/<id>.json hold tiles and placed objects
Replaces the .txt maps plus the Excel FieldObjects sheet (markers) with
one JSON file per map: tiles, P/S positions and objects with x/y. The
converter validates floor positions, duplicate ids, refs, patrol paths
against walls, schedules and conditions. Runtime map data is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -20,11 +20,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyParts" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAttacks" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldObjects" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survival" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampActions" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revivals" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survival" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampActions" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revivals" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1196,498 +1195,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>object_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>map_id</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>marker</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ref</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>patrol</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>fo_enemy1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>enemy</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>enemy_test</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>적 A (테스트)</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>right 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>fo_enemy2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>enemy</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>enemy_test</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>적 A (테스트)</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>down 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>fo_look1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>investigate</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>spot_b</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>조사 지점 1</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>조사 텍스트 1 (테스트)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>fo_look2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>d</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>investigate</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>spot_charm</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>조사 지점 2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>조사 텍스트 2 (테스트, 부활 아이템)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>fo_look3</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>investigate</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>spot_empty</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>조사 지점 3</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>조사 텍스트 3 (테스트, 빈 탐색)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>fo_npc1</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>npc</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>fd_npc1_a</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>NPC 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>fo_npc2</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>npc</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>fd_npc2_a</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>NPC 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>fo_camp</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>basecamp</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>c</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>camp</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>베이스캠프 거점</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>fo_to_field</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>basecamp</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>exit</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>탐험 지역으로</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>fo_to_camp</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>exit</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>basecamp</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>베이스캠프로</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>fo_supply</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>test_field</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>f</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>investigate</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>spot_supply</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>보급 상자</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>조사 텍스트 4 (테스트, 음식·물)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>fo_cat</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>basecamp</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>k</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>npc</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>fd_cat_a</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>고양이</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>06:00-12:00, 20:00-23:00</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1856,7 +1363,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2010,7 +1517,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2112,13 +1619,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A62"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -2131,6 +1638,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -2166,6 +1674,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -2208,6 +1717,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -2257,6 +1767,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -2306,6 +1817,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -2348,20 +1860,9 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>[탐험] 맵 모양: tools/maps/&lt;map_id&gt;.txt  (# 벽, . 바닥, P 시작 위치, 그 밖의 글자 = FieldObjects 의 marker)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>FieldObjects: type enemy(ref=enemy_id, patrol='right 4' 처럼 방향+칸수 왕복) / investigate(text 표시, ref=Loot spot_id 면 아이템 굴림)</t>
-        </is>
-      </c>
-    </row>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
@@ -2369,6 +1870,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
@@ -2376,13 +1878,7 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>FieldObjects type=npc, ref=필드 대화 시작 노드. 말을 걸 때마다 시작 노드부터 (조건·플래그로 내용 분기)</t>
-        </is>
-      </c>
-    </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
@@ -2390,6 +1886,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
@@ -2404,20 +1901,8 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>[베이스캠프] CampActions: 베이스캠프 거점(FieldObjects type=camp)에서 고르는 행동. minutes = 걸리는 시간, kind=save 는 저장</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>FieldObjects type=exit: ref = 이동할 맵 이름. 도착하면 그 맵의 P 위치</t>
-        </is>
-      </c>
-    </row>
+    <row r="49"/>
+    <row r="50"/>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
@@ -2425,13 +1910,8 @@
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>[저장] 베이스캠프에서만. 고양이(FieldObjects condition 이 참일 때만 나타남)에게 효과 save 로 저장하거나, 잠자기(CampActions kind=sleep)로 자고 나면 저장</t>
-        </is>
-      </c>
-    </row>
+    <row r="52"/>
+    <row r="53"/>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
@@ -2446,20 +1926,9 @@
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>FieldObjects.condition: 맵에 들어올 때 참이어야 물체가 나타남 (비우면 항상)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>FieldObjects.schedule (npc): 하루 중 있는 시간대 '06:00-12:00, 20:00-23:00'. 자정 넘김 '22:00-02:00' 가능. 시간이 흐르면 나타나고 사라짐</t>
-        </is>
-      </c>
-    </row>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
@@ -2474,17 +1943,18 @@
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>맵 글자 S: 새 회차 시작 위치 (Config start_map 의 맵). 없으면 P</t>
-        </is>
-      </c>
-    </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
           <t>Config save_slots: 저장 슬롯 수. 잠에서 깨거나 효과 save(고양이)로 저장할 때 슬롯을 고름</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>[맵] 맵 모양과 맵 위 물체(적·조사·NPC·거점·출구)는 Godot '맵' 탭에서 편집 → tools/maps/&lt;맵ID&gt;.json</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Limb-restoration trade mechanics: cut:/count: conditions, restore: effect
- Condition cut:<part>|any (severed non-vital limb), count:death|run (world records, §11)
- Effect restore:<part>|all puts severed limbs back at full HP (§10); cost is paid by the
  other effects in the same choice
- Converter checks part ids (must be non-vital PlayerParts) and count names
- Tests: test_expr 79, test_survival 52

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -1625,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A63"/>
+  <dimension ref="A1:A67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1638,7 +1638,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1674,7 +1673,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1717,7 +1715,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -1767,7 +1764,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -1817,7 +1813,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -1860,9 +1855,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
@@ -1870,7 +1862,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
@@ -1878,7 +1869,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
@@ -1886,7 +1876,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
@@ -1901,8 +1890,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50"/>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
@@ -1910,8 +1897,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
-    <row r="53"/>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
@@ -1926,9 +1911,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
@@ -1943,7 +1925,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
@@ -1955,6 +1936,27 @@
       <c r="A63" t="inlineStr">
         <is>
           <t>[맵] 맵 모양과 맵 위 물체(적·조사·NPC·거점·출구)는 Godot '맵' 탭에서 편집 → tools/maps/&lt;맵ID&gt;.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>[사지 복구 거래 §10] 조건 cut:left_arm (그 팔다리가 잘렸나) / cut:any (하나라도). 대상은 PlayerParts 의 vital 이 아닌 부위</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>효과 restore:left_arm / restore:all (잘린 팔다리를 최대 HP로 복구). 대가는 같은 effects 에 함께 적어 즉시 지불 (예: item:-relic;restore:left_arm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>조건 count:death&gt;=1 / count:run&gt;=2 (월드 기록: 사망 횟수(부활 포함)·회차 수). 초월체의 '또 왔네' 분기용</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Combat choice type: start a fight from a field dialogue choice
- Choices.type=combat, check=enemy_id (field dialogues only). Win -> effects/next_node,
  flee -> fail_effects/fail_next, lose -> dialogue closes and the field runs death/revival
- StoryRunner.combat_requested / finish_combat; field hides the dialogue during the fight
- Choice button shows "[전투] text (enemy name)"; dialogue editor gets the type, enemy picker
  and a flee port; switching back to normal/item clears check/fail fields
- Converter checks enemy_id, field-only, and a flee exit
- Dummy: npc2 choice fdc7. Tests: test_story 68, field_smoke flee/win/lose

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -1625,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A67"/>
+  <dimension ref="A1:A68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1957,6 +1957,13 @@
       <c r="A67" t="inlineStr">
         <is>
           <t>조건 count:death&gt;=1 / count:run&gt;=2 (월드 기록: 사망 횟수(부활 포함)·회차 수). 초월체의 '또 왔네' 분기용</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Choices.type=combat (필드 대화 전용): check=enemy_id. 이기면 effects·next_node, 도주하면 fail_effects·fail_next, 지면 대화가 끝나고 사망 처리(Revivals)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Combat screen redesign: enemy name/image, body status, text box, 3 actions
- Layout from the mockup: enemy name top-left with underline, enemy image in the
  centre (Enemies.image, silhouette when empty), "내 상태" body figure bottom-left,
  text box bottom-centre (messages + part choices), action buttons 공격/아이템/도주
- Attack: enemy parts listed as choices in the text box (HP, hit chance) + cancel
- Item: opens the inventory; consumables use StoryRunner.use_item_in_combat, effects
  reach the in-combat body; Config combat_item_uses_turn (default 1)
- Flee: d100 roll animation, success if roll <= Enemies.flee_chance (fallback Config)
- Defend button removed from the screen (rule code kept)
- Converter: optional Enemies columns flee_chance (0-100) and image (res:// file must exist)
- Tests: test_combat 38, combat_smoke rewritten (attack, item, flee fail/success, death)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -761,7 +761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -779,6 +779,16 @@
           <t>name</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>flee_chance</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -790,6 +800,9 @@
         <is>
           <t>적 A (테스트)</t>
         </is>
+      </c>
+      <c r="C2" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1625,7 +1638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A68"/>
+  <dimension ref="A1:A69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1964,6 +1977,13 @@
       <c r="A68" t="inlineStr">
         <is>
           <t>Choices.type=combat (필드 대화 전용): check=enemy_id. 이기면 effects·next_node, 도주하면 fail_effects·fail_next, 지면 대화가 끝나고 사망 처리(Revivals)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Enemies.flee_chance: 도주 성공률 % (주사위 1~100 이 이 값 이하면 성공, 비우면 Config combat_flee_chance). Enemies.image: 전투 화면 그림 res:// 경로 (비우면 도형)</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4427,6 +4447,21 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>combat_item_uses_turn</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>전투 중 아이템 사용이 턴을 쓰는지 (1 = 씀, 0 = 안 씀). TODO 기획 7.1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Grid inventory (I), equipment window (Q) with stats tab, bags and carry weight
- Inventory is a grid of cells; slot count = Config inventory_slots + bag_slots of equipped items
- Equipment window: equip tab (EquipSlots from player.xlsx) and stats tab (body status on top,
  six abilities as a hexagon). Open both and drag items between them to equip/unequip;
  right-click in the inventory equips, right-click on a slot unequips
- Items get weight / equip_slot / bag_slots (item.xlsx); carry weight slows the player past
  Config carry_heavy_weight and stops them at carry_max_weight (placeholder values, TODO)
- Equipped items count for has:, dice bonuses and item:- effects; saved with the run
- Dummy data: small_bag (+4 slots) at spot_charm, knife equips as weapon
- Tests: test_equipment (17), equipment_smoke; ui/basecamp smoke updated for grid cell text

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Episodes" sheetId="1" state="visible" r:id="rId1"/>
@@ -608,7 +608,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -644,7 +643,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -687,7 +685,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -737,7 +734,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
@@ -787,7 +783,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
@@ -830,9 +825,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -840,7 +832,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -848,7 +839,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
@@ -856,7 +846,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
@@ -871,8 +860,6 @@
         </is>
       </c>
     </row>
-    <row r="50"/>
-    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -880,8 +867,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
-    <row r="54"/>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
@@ -896,9 +881,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -913,7 +895,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
@@ -928,7 +909,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -964,7 +944,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
@@ -2416,7 +2395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2834,6 +2813,66 @@
       <c r="C27" t="inlineStr">
         <is>
           <t>전투 중 아이템 사용이 턴을 쓰는지 (1 = 씀, 0 = 안 씀). TODO 기획 7.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>carry_max_weight</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>30</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>들 수 있는 최대 무게. 이 이상이면 움직일 수 없음 (TODO 기획: 임시값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>carry_heavy_weight</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>20</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>이 무게 이상이면 이동 속도가 느려짐 (TODO 기획: 임시값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>carry_heavy_speed_mult</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>무거울 때 이동 속도 배율 (TODO 기획: 임시값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ability_chart_max</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>능력치 육각형 그래프의 바깥 끝 값 (표시용)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Equipment slots as in the mockup (bag, head, hands, body, legs); 4 base slots; hands hold any item
EquipSlots get kind/col/row; items name a kind in equip_slot; hand slots take any item and do not use inventory slots. Config inventory_slots 4. Tests updated to use the configured slot count.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2427,11 +2427,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>인벤토리 칸 수</t>
+          <t>가방이 없을 때 소지품 칸 수 (손에 든 것은 안 셈)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Status effects and the new stats tab layout
StatusEffects sheet (content.xlsx); effects status:+id/-id and condition status:id in the runtime, converter and editor pickers; saved with the run. Stats tab: body on the left, status list (hover shows description) top right, ability hexagon bottom right.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -11,11 +11,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choices" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endings" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abilities" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survival" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampActions" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revivals" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StatusEffects" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survival" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampActions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revivals" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -588,7 +589,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A73"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>revive_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>effects</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>rv_charm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>부활 부적</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>has:charm</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>item:-charm</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>부활 텍스트 1 (테스트, 아이템으로 부활)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>rv_hana</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>초월체의 보호</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>flag:hana_protect</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>clearflag:hana_protect</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>부활 텍스트 2 (테스트, 초월체가 부활시킴)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -955,6 +1058,13 @@
       <c r="A73" t="inlineStr">
         <is>
           <t>능력치 열: walk_speed 걷기·run_speed 달리기 (필드 칸/초. 플레이어는 Shift 로 달림, 적은 순찰=걷기·추격=달리기), strength 근력, endurance 지구력, intelligence 지능, health 건강, mental 정신력, divinity 신성력 (스킬용, TODO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>[상태이상] StatusEffects: status_id, name, description (장비창 능력치 탭에서 이름에 마우스를 올리면 설명). 효과 status:+bleeding 걸기 / status:-bleeding 풀기, 조건 status:bleeding. 실제 효과는 아직 없음 (TODO 기획)</t>
         </is>
       </c>
     </row>
@@ -2395,6 +2505,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>status_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>bleeding</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>출혈</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>(테스트) 효과 설명 — 기획 TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>nausea</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>매스꺼움</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>(테스트) 효과 설명 — 기획 TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>panic</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>공황</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>(테스트) 효과 설명 — 기획 TODO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
@@ -2881,7 +3078,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3053,7 +3250,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3205,106 +3402,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>revive_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>effects</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>rv_charm</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>부활 부적</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>has:charm</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>item:-charm</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>부활 텍스트 1 (테스트, 아이템으로 부활)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>rv_hana</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>초월체의 보호</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>flag:hana_protect</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>clearflag:hana_protect</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>부활 텍스트 2 (테스트, 초월체가 부활시킴)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Map travel: passages, transit points, map edges, move effect and arrival points
New map objects passage (step on), transit (E, e.g. ladder) and arrive (named arrival point); exits, passages, transits and map edges pick a target map and arrival point (P if empty). Effect move:map[@arrive] travels after the dialogue ends. Map editor tools, edge settings and arrival pickers; converter checks targets. Dummy map test_travel, basecamp arrival bc_gate. Test travel_smoke.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -691,7 +691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A74"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1065,6 +1065,13 @@
       <c r="A74" t="inlineStr">
         <is>
           <t>[상태이상] StatusEffects: status_id, name, description (장비창 능력치 탭에서 이름에 마우스를 올리면 설명). 효과 status:+bleeding 걸기 / status:-bleeding 풀기, 조건 status:bleeding. 실제 효과는 아직 없음 (TODO 기획)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>[맵 이동] 효과 move:map_id (그 맵의 P) / move:map_id@arrive_id (그 맵의 도착 지점). 필드 대화·아이템·거점 행동에서만, 대화 중이면 대화가 끝난 뒤 이동</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dialogue editor v1.0: script blocks with multiple pages, typing, new layout
- Node pages (narration / bubble / system) with speed, inline {w=} pauses, auto advance;
  nodes without pages still play as one page (old files unchanged on save)
- Play screen types text; first input shows the page, next input advances
- Editor: explorer (list, search all dialogues, palette), script panel under the graph,
  foldable inspector, check panel with click-to-jump, undo/redo, copy/paste/duplicate,
  drag-to-empty creates a card, fold, auto arrange, unsaved prompt, minimap
- Converter checks pages, adds warnings; Config text_speed_* keys
- Tests: test_script_pages, dialogue editor smoke on fixtures

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2599,7 +2599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3077,6 +3077,68 @@
       <c r="C31" t="inlineStr">
         <is>
           <t>능력치 육각형 그래프의 바깥 끝 값 (표시용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>text_speed_default</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>대사 기본 출력 속도: instant / slow / normal / fast (대화 파일·페이지에서 바꿀 수 있음). TODO 기획 §10.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>text_speed_slow</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>15</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>느림: 초당 글자 수 (임시값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>text_speed_normal</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>35</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>보통: 초당 글자 수 (임시값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>text_speed_fast</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>70</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>빠름: 초당 글자 수 (임시값)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Traits sheet in player.xlsx and status effects in new status.xlsx
- player.xlsx Traits: 40 creation trait candidates (polarity, signed points,
  category, conflicts, selectable, state) from the character creation spec v0.1
- status.xlsx StatusEffects: 4 confirmed + 8 candidate statuses with scope,
  tick fields and death cause; undecided values left blank. Removed from content.xlsx.
- Converter validates both; unknown trait names are warnings
- Dummy status panic renamed to panic_disorder

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -11,12 +11,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choices" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endings" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abilities" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StatusEffects" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survival" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampActions" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revivals" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survival" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampActions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revivals" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -589,108 +588,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>revive_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>effects</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>rv_charm</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>부활 부적</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>has:charm</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>item:-charm</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>부활 텍스트 1 (테스트, 아이템으로 부활)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>rv_hana</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>초월체의 보호</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>flag:hana_protect</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>clearflag:hana_protect</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>부활 텍스트 2 (테스트, 초월체가 부활시킴)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:A75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
@@ -707,10 +604,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>엑셀 파일 나눔: player.xlsx (Player·PlayerParts) / npc.xlsx (Npcs·NpcParts·NpcAttacks) / item.xlsx (Items·Loot) / 나머지는 이 파일</t>
-        </is>
-      </c>
-    </row>
+          <t>엑셀 파일 나눔: player.xlsx (Player·PlayerParts·EquipSlots·Traits) / npc.xlsx (Npcs·NpcParts·NpcAttacks) / item.xlsx (Items·Loot) / status.xlsx (StatusEffects) / 나머지는 이 파일</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -746,6 +644,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -788,6 +687,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -837,6 +737,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
@@ -886,6 +787,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
@@ -928,6 +830,9 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -935,6 +840,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -942,6 +848,7 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
@@ -949,6 +856,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
@@ -963,6 +871,8 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
+    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -970,6 +880,8 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
+    <row r="54"/>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
@@ -984,6 +896,9 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -998,6 +913,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
@@ -1012,6 +928,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -1047,6 +964,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
@@ -2512,93 +2430,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>status_id</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>bleeding</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>출혈</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>(테스트) 효과 설명 — 기획 TODO</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>nausea</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>매스꺼움</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>(테스트) 효과 설명 — 기획 TODO</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>panic</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>공황</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>(테스트) 효과 설명 — 기획 TODO</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
@@ -3147,7 +2978,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3319,7 +3150,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3471,4 +3302,106 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>revive_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>effects</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>rv_charm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>부활 부적</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>has:charm</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>item:-charm</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>부활 텍스트 1 (테스트, 아이템으로 부활)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>rv_hana</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>초월체의 보호</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>flag:hana_protect</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>clearflag:hana_protect</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>부활 텍스트 2 (테스트, 초월체가 부활시킴)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Character creation with trait points, persistent traits, traits tab
- Creation screen: start points 5 (Config creation_start_points), positive traits
  cost / negative traits give points, blocked reasons, confirm summary
- Title: new game -> creation; once created, new run keeps the character,
  "new game" resets world record and traits (save slots kept)
- GameState.owned_traits kept across runs (world save) and in run saves;
  loading a slot restores that slot's traits (spec 5.4 option B)
- Effects trait:+id / trait:-id with notice; picker rows in the editors
- Equipment window third tab: owned traits split positive / negative

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -608,7 +608,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -644,7 +643,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -687,7 +685,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -737,7 +734,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
@@ -787,7 +783,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
@@ -830,9 +825,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -840,7 +832,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -848,7 +839,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
@@ -856,7 +846,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
@@ -871,8 +860,6 @@
         </is>
       </c>
     </row>
-    <row r="50"/>
-    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -880,8 +867,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
-    <row r="54"/>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
@@ -896,9 +881,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -913,7 +895,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
@@ -928,7 +909,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -964,7 +944,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
@@ -2430,7 +2409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2970,6 +2949,21 @@
       <c r="C35" t="inlineStr">
         <is>
           <t>빠름: 초당 글자 수 (임시값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>creation_start_points</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>캐릭터 생성 시작 포인트 (긍정 특성은 소비, 부정 특성은 획득). 기획 §2.2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monster kind and talking during combat
- Npcs kind = monster / npc; map enemies that are not monsters warn,
  map tab lists monsters first
- Combat action panel: 공격 / 특수 / 대화 / 아이템 / 도주. 대화 opens the
  opponent's NPC dialogue over the combat screen (NPC or monster)
- Condition combat:any / combat:<npc_id>, effect endcombat:win / endcombat:flee;
  a fight choice inside a combat talk returns to the fight
- Runner state saved and restored around the combat talk; hidden dialogue
  screens ignore runner signals
- Dummy dialogue monster_test (enemy_test), tests updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2409,7 +2409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2964,6 +2964,21 @@
       <c r="C36" t="inlineStr">
         <is>
           <t>캐릭터 생성 시작 포인트 (긍정 특성은 소비, 부정 특성은 획득). 기획 §2.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>combat_talk_uses_turn</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>전투 중 '대화'가 턴을 쓰나 (1 = 대화 뒤 적 차례, 0 = 다시 내 차례). TODO 기획</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cutscene sound, facing, skip button and opening cutscene
- Steps sound / music / music_off with a Sound autoload (BGM loops across
  scenes, files loaded directly when not imported); listen button in the card
- Facing: NPCs and the player show a facing mark, walking faces the move,
  step face, map NPC starting face
- Skip button (and Esc) during cutscenes: steps finish instantly, text pages
  advance on their own, stops at a choice or the end
- Opening cutscene: Config opening_dialogue plays once after character creation
  (dummy opening.json); converter checks audio files, face and the opening node
- Dummy sounds audio/sfx/test_beep.wav, audio/bgm/test_loop.wav; tests extended

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2409,7 +2409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2979,6 +2979,23 @@
       <c r="C37" t="inlineStr">
         <is>
           <t>전투 중 '대화'가 턴을 쓰나 (1 = 대화 뒤 적 차례, 0 = 다시 내 차례). TODO 기획</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>opening_dialogue</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>opening_in</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>새 게임(캐릭터 생성 직후) 오프닝 컷신의 첫 노드. 비우면 없음 (지금은 테스트용 opening.json)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Opening chosen in the dialogue editor; dialogues without an NPC
- Start card checkbox "게임 오프닝으로 쓰기" (dialogue file opening: true);
  converter resolves it when Config has no opening_dialogue, errors on two
- New dialogue dialog: "NPC 없음 (오프닝·이벤트 컷신)"; list marks the opening

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A75"/>
+  <dimension ref="A1:A77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -969,6 +969,14 @@
       <c r="A75" t="inlineStr">
         <is>
           <t>[맵 이동] 효과 move:map_id (그 맵의 P) / move:map_id@arrive_id (그 맵의 도착 지점). 필드 대화·아이템·거점 행동에서만, 대화 중이면 대화가 끝난 뒤 이동</t>
+        </is>
+      </c>
+    </row>
+    <row r="76"/>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>오프닝 컷신: 대화 에디터에서 대화 시작 카드 → '🎬 게임 오프닝으로 쓰기' 체크 (대화 하나만). 엑셀로 정하려면 Config 에 opening_dialogue = 첫 노드 ID 줄을 추가 (그쪽이 먼저)</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2979,23 +2987,6 @@
       <c r="C37" t="inlineStr">
         <is>
           <t>전투 중 '대화'가 턴을 쓰나 (1 = 대화 뒤 적 차례, 0 = 다시 내 차례). TODO 기획</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>opening_dialogue</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>opening_in</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>새 게임(캐릭터 생성 직후) 오프닝 컷신의 첫 노드. 비우면 없음 (지금은 테스트용 opening.json)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Death causes: Excel list of death messages shown on the death screen
content.xlsx DeathCauses (cause_id, name, text). The death panel shows
the cause's text, or "{name}(으)로 인해 사망했습니다." when text is empty.
Causes: combat loss, a survival value with death_cause reaching 0
(hunger = starvation, thirst = dehydration), and the effect die:cause_id.
Revival raises those survival values to Config revive_survival_floor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -15,7 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survival" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CampActions" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revivals" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DeathCauses" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_help" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -588,6 +589,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>cause_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>starvation</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>굶주림</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>굶어 죽었습니다.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Survival hunger 가 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dehydration</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>탈수</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>탈수로 죽었습니다.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Survival thirst 가 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>combat</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{enemy}의 공격</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>전투에서 짐. text 를 비우면 '{name}(으)로 인해 사망했습니다.' ({enemy} = 상대 이름)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>알 수 없는 원인</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>원인을 모를 때</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
@@ -2416,7 +2539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3001,6 +3124,21 @@
       <c r="C38" t="inlineStr">
         <is>
           <t>픽셀아트 타일 한 칸의 그림 크기 (px). 게임에서는 field_tile(80) 로 늘려 그림 (5배)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>revive_survival_floor</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>10</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>부활할 때 생존 수치가 이보다 낮으면 이 값으로 (0 이면 바로 다시 죽으므로). 임시값 TODO 기획</t>
         </is>
       </c>
     </row>
@@ -3015,13 +3153,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="2"/>
     <col width="7" customWidth="1" min="3" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3055,6 +3194,11 @@
           <t>warn</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>death_cause</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3079,6 +3223,11 @@
       <c r="F2" t="n">
         <v>30</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>starvation</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3102,6 +3251,11 @@
       </c>
       <c r="F3" t="n">
         <v>30</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>dehydration</t>
+        </is>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Monster AI phase 6 (field): hearing, flashlight sight, map-to-map pursuit, debug control
- Running (every noise_interval) and opening/closing doors make noise;
  BT monsters within the radius hear it (UpdateNoise service). Template
  BT_02_HearAndSearch investigates sounds.
- Holding a flashlight multiplies monster sight (ai_flashlight_sight_mult).
- Monsters chasing the player follow through doors after ai_follow_delay
  seconds and stay in that map (field_state followers / gone); per-monster
  'follow' off in the map editor.
- Field accepts monster_ai pause / step / breakpoints messages from the
  editor; a breakpoint pauses all monsters.
Config values are placeholders (TODO design).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -675,7 +675,6 @@
           <t>{enemy}의 공격</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>전투에서 짐. text 를 비우면 '{name}(으)로 인해 사망했습니다.' ({enemy} = 상대 이름)</t>
@@ -693,7 +692,6 @@
           <t>알 수 없는 원인</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>원인을 모를 때</t>
@@ -2539,7 +2537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3139,6 +3137,96 @@
       <c r="C39" t="inlineStr">
         <is>
           <t>부활할 때 생존 수치가 이보다 낮으면 이 값으로 (0 이면 바로 다시 죽으므로). 임시값 TODO 기획</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>noise_run_radius</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>6</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>몬스터 AI 청각: 달리면 이 반경(칸) 안의 BT 몬스터가 들음. 임시값 TODO 기획</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>noise_door_radius</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>몬스터 AI 청각: 문을 여닫으면 이 반경(칸). 임시값 TODO 기획</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>noise_interval</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>달리는 동안 소리를 내는 간격(초). 임시값</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ai_flashlight_sight_mult</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>손전등을 들고 있으면 몬스터 시야 × 이 값. 임시값 TODO 기획</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ai_follow_enabled</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1 = 쫓던 몬스터가 다른 맵까지 따라옴 (몬스터별로 맵 에디터 '따라오기' 끔 가능)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ai_follow_delay</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>따라 들어오기까지 초. 임시값 TODO 기획</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Combat with up to 3 monsters at once
Combat logic keeps a list of foes (setup_many, select, alive, defeated,
withdraw); a single foe behaves as before. When a fight starts with a
monster, other monsters chasing the player within combat_join_radius join,
nearest first, up to combat_max_enemies (3); NPCs always fight alone. The
combat screen draws each foe side by side with names, asks which foe to
attack or talk to, and lets every living foe attack in turn. After the
fight only defeated or withdrawn foes leave the map. Also: monsters only
walk straight when their whole body clears walls (no snagging on corners),
and finishing a fight twice is ignored.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2537,7 +2537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3227,6 +3227,36 @@
       <c r="C45" t="inlineStr">
         <is>
           <t>따라 들어오기까지 초. 임시값 TODO 기획</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>combat_max_enemies</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>한 번에 함께 싸우는 몬스터 최대 수 (NPC 는 늘 혼자)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>combat_join_radius</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>8</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>전투가 시작될 때 이 반경(칸) 안에서 쫓아오던 몬스터가 함께 들어옴. 임시값 TODO 기획</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
3/4 top-down view (wall front faces) and player sprite
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2537,7 +2537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3257,6 +3257,68 @@
       <c r="C47" t="inlineStr">
         <is>
           <t>전투가 시작될 때 이 반경(칸) 안에서 쫓아오던 몬스터가 함께 들어옴. 임시값 TODO 기획</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>player_sprite</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>res://art/characters/player.png</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>플레이어 캐릭터 그림 (프레임을 가로로 이어 붙인 PNG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>player_sprite_frames</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>그림 프레임 수 (걷는 동안 번갈아)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>player_sprite_frame_time</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>프레임 하나의 초 (달리면 0.6배)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>character_scale</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>캐릭터 그림 배율. 0 = 타일과 같은 픽셀 밀도 (field_tile / tile_art_px)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Windows with daylight and curtains; doors placed on walls open the wall
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2537,7 +2537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3319,6 +3319,36 @@
       <c r="C51" t="inlineStr">
         <is>
           <t>캐릭터 그림 배율. 0 = 타일과 같은 픽셀 밀도 (field_tile / tile_art_px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>window_light_energy</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>창문으로 들어오는 햇빛 밝기 (한낮 기준, 시간대에 따라 실외 sun_energy 비율로 줄어듦·밤엔 꺼짐) — 임시</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>window_light_radius</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>창문 빛이 닿는 거리 (칸) — 임시</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Church map (back wall, windows, indoor), basecamp map, Config (basecamp_map, vignette) and converted data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="13005" yWindow="1320" windowWidth="22635" windowHeight="18480" tabRatio="600" firstSheet="1" activeTab="8" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Episodes" sheetId="1" state="visible" r:id="rId1"/>
@@ -49,7 +49,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -590,7 +594,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -2436,7 +2440,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -2537,7 +2541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2859,7 +2863,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>basecamp</t>
+          <t>new_america_in_church</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3349,6 +3353,53 @@
       <c r="C53" t="inlineStr">
         <is>
           <t>창문 빛이 닿는 거리 (칸) — 임시</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>vignette_strength</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>화면 가장자리 어둠 세기 (0 = 끔 ~ 1 = 가장자리 완전히 검게) — 임시</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>vignette_inner</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>어두워지기 시작하는 거리 (0 = 화면 가운데부터 ~ 1 = 가장자리 근처부터)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>vignette_color</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>#000000</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>비네트 색 (#RRGGBB)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wandering NPCs (radius or route), Config speed/pauses; converter warns on overlapping NPC schedules
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2541,7 +2541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3400,6 +3400,51 @@
       <c r="C56" t="inlineStr">
         <is>
           <t>비네트 색 (#RRGGBB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>npc_wander_speed</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>돌아다니는 NPC 걷는 속도 (칸/초) — 임시</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>npc_wander_wait_min</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>돌아다니는 NPC 쉬는 시간 최소 (초) — 임시</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>npc_wander_wait_max</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>6</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>돌아다니는 NPC 쉬는 시간 최대 (초) — 임시</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Quarter view (isometric) game screen: diamond floors, wall blocks, iso proxies for actors and objects, screen-relative movement (logic unchanged)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -2541,7 +2541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3445,6 +3445,38 @@
       <c r="C59" t="inlineStr">
         <is>
           <t>돌아다니는 NPC 쉬는 시간 최대 (초) — 임시</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>view_mode</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>iso</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>게임 화면: iso = 쿼터뷰(아이소메트릭, 마름모) / topdown = 비스듬한 탑뷰 (규칙·맵은 같음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>iso_wall_height</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>120</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>쿼터뷰 벽 블록 높이 (화면 px, 한 칸 = 80) — 임시</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Work-in-progress content: New America village/church maps, intro cutscene and art, world layout, sheet edits (start map, player name), remove city map and old opening dummy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sheets/content.xlsx
+++ b/tools/sheets/content.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="13005" yWindow="1320" windowWidth="22635" windowHeight="18480" tabRatio="600" firstSheet="1" activeTab="8" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="13005" yWindow="1320" windowWidth="22635" windowHeight="18480" tabRatio="600" firstSheet="1" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Episodes" sheetId="1" state="visible" r:id="rId1"/>
@@ -553,7 +553,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>char_t2</t>
+          <t>char_t1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -733,6 +733,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -768,6 +769,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -810,6 +812,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -859,6 +862,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
@@ -908,6 +912,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
@@ -950,6 +955,9 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
@@ -957,6 +965,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -964,6 +973,7 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
@@ -971,6 +981,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
@@ -985,6 +996,8 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
+    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -992,6 +1005,8 @@
         </is>
       </c>
     </row>
+    <row r="53"/>
+    <row r="54"/>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
@@ -1006,6 +1021,9 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -1020,6 +1038,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
@@ -1034,6 +1053,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -1069,6 +1089,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
@@ -1097,6 +1118,7 @@
         </is>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
@@ -1306,7 +1328,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>char_t2</t>
+          <t>char_t1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2846,7 +2868,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>test_field</t>
+          <t>new_america_in_church</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>